<commit_message>
docs(roadmap): flip v1.0 Clinical Safety rows 2-3 to completed
PR #282 (v1.0 / Clinical Safety / CDS Hooks expansion + Drug-drug
interaction check) is now on main (commit 472352cd) and develop
(commit 7917ff58), so both rows graduate from "started" to
"completed" per docs/roadmap.md status definition ("Shipped. The
deliverable described in the row is verifiable on the listed
branch").

Regenerated docs/roadmap.xlsx from the updated CSV — both rows now
render with the green "completed" tint.
</commit_message>
<xml_diff>
--- a/docs/roadmap.xlsx
+++ b/docs/roadmap.xlsx
@@ -52,7 +52,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFE699"/>
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -611,7 +611,7 @@
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>started</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>started</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs(roadmap): start v1.0 row 7 — Idle session timeout (server-side)
Picks up the next v1.0 / Security row after CDS Hooks expansion + DDI
shipped (rows 2-3 → completed in e2fe6c91).

Plan: track last-activity in Redis (mirrors the
RedisTokenBlacklistService pattern: hms:idle:user:<uuid> TTL'd at the
configured idle window), reject requests after 15 min idle from both
the legacy JwtAuthenticationFilter AND the OIDC
KeycloakHospitalContextFilter, gate the refresh endpoint, carve out
service-to-server clients (FHIR / HL7 MLLP / CDS Hooks / DHIS2 ADX /
partner pharmacy SMS webhook). Fail-open with throttled WARN + Micro-
meter counter on Redis outage so a Redis blip does not lock every
clinician out.

Unblocks row 8 (Keycloak Phase C cutover, OIDC_REQUIRED=true).
</commit_message>
<xml_diff>
--- a/docs/roadmap.xlsx
+++ b/docs/roadmap.xlsx
@@ -33,7 +33,7 @@
       <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +58,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE699"/>
       </patternFill>
     </fill>
     <fill>
@@ -107,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -134,6 +139,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -869,9 +877,9 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>started</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
@@ -1193,7 +1201,7 @@
       </c>
     </row>
     <row r="14" ht="38" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1245,7 +1253,7 @@
       </c>
     </row>
     <row r="15" ht="38" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1297,7 +1305,7 @@
       </c>
     </row>
     <row r="16" ht="38" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1349,7 +1357,7 @@
       </c>
     </row>
     <row r="17" ht="38" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1401,7 +1409,7 @@
       </c>
     </row>
     <row r="18" ht="38" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1453,7 +1461,7 @@
       </c>
     </row>
     <row r="19" ht="38" customHeight="1">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1505,7 +1513,7 @@
       </c>
     </row>
     <row r="20" ht="38" customHeight="1">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1557,7 +1565,7 @@
       </c>
     </row>
     <row r="21" ht="38" customHeight="1">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1609,7 +1617,7 @@
       </c>
     </row>
     <row r="22" ht="38" customHeight="1">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1661,7 +1669,7 @@
       </c>
     </row>
     <row r="23" ht="38" customHeight="1">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1713,7 +1721,7 @@
       </c>
     </row>
     <row r="24" ht="38" customHeight="1">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1765,7 +1773,7 @@
       </c>
     </row>
     <row r="25" ht="38" customHeight="1">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1817,7 +1825,7 @@
       </c>
     </row>
     <row r="26" ht="38" customHeight="1">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1869,7 +1877,7 @@
       </c>
     </row>
     <row r="27" ht="38" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -1921,7 +1929,7 @@
       </c>
     </row>
     <row r="28" ht="38" customHeight="1">
-      <c r="A28" s="7" t="inlineStr">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -1973,7 +1981,7 @@
       </c>
     </row>
     <row r="29" ht="38" customHeight="1">
-      <c r="A29" s="7" t="inlineStr">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -2025,7 +2033,7 @@
       </c>
     </row>
     <row r="30" ht="38" customHeight="1">
-      <c r="A30" s="7" t="inlineStr">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -2077,7 +2085,7 @@
       </c>
     </row>
     <row r="31" ht="38" customHeight="1">
-      <c r="A31" s="7" t="inlineStr">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -2129,7 +2137,7 @@
       </c>
     </row>
     <row r="32" ht="38" customHeight="1">
-      <c r="A32" s="7" t="inlineStr">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -2181,7 +2189,7 @@
       </c>
     </row>
     <row r="33" ht="38" customHeight="1">
-      <c r="A33" s="7" t="inlineStr">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -2233,7 +2241,7 @@
       </c>
     </row>
     <row r="34" ht="38" customHeight="1">
-      <c r="A34" s="7" t="inlineStr">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -2285,7 +2293,7 @@
       </c>
     </row>
     <row r="35" ht="38" customHeight="1">
-      <c r="A35" s="7" t="inlineStr">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -2337,7 +2345,7 @@
       </c>
     </row>
     <row r="36" ht="38" customHeight="1">
-      <c r="A36" s="7" t="inlineStr">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -2389,7 +2397,7 @@
       </c>
     </row>
     <row r="37" ht="38" customHeight="1">
-      <c r="A37" s="7" t="inlineStr">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -2441,7 +2449,7 @@
       </c>
     </row>
     <row r="38" ht="38" customHeight="1">
-      <c r="A38" s="7" t="inlineStr">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -2493,7 +2501,7 @@
       </c>
     </row>
     <row r="39" ht="38" customHeight="1">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="A39" s="9" t="inlineStr">
         <is>
           <t>oos</t>
         </is>
@@ -2533,7 +2541,7 @@
           <t>â€”</t>
         </is>
       </c>
-      <c r="I39" s="8" t="inlineStr">
+      <c r="I39" s="9" t="inlineStr">
         <is>
           <t>deferred</t>
         </is>
@@ -2545,7 +2553,7 @@
       </c>
     </row>
     <row r="40" ht="38" customHeight="1">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="A40" s="9" t="inlineStr">
         <is>
           <t>oos</t>
         </is>
@@ -2585,7 +2593,7 @@
           <t>â€”</t>
         </is>
       </c>
-      <c r="I40" s="8" t="inlineStr">
+      <c r="I40" s="9" t="inlineStr">
         <is>
           <t>deferred</t>
         </is>
@@ -2597,7 +2605,7 @@
       </c>
     </row>
     <row r="41" ht="38" customHeight="1">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="A41" s="9" t="inlineStr">
         <is>
           <t>oos</t>
         </is>
@@ -2637,7 +2645,7 @@
           <t>â€”</t>
         </is>
       </c>
-      <c r="I41" s="9" t="inlineStr">
+      <c r="I41" s="10" t="inlineStr">
         <is>
           <t>dropped</t>
         </is>
@@ -2649,7 +2657,7 @@
       </c>
     </row>
     <row r="42" ht="38" customHeight="1">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="A42" s="9" t="inlineStr">
         <is>
           <t>oos</t>
         </is>
@@ -2689,7 +2697,7 @@
           <t>â€”</t>
         </is>
       </c>
-      <c r="I42" s="9" t="inlineStr">
+      <c r="I42" s="10" t="inlineStr">
         <is>
           <t>dropped</t>
         </is>
@@ -2701,7 +2709,7 @@
       </c>
     </row>
     <row r="43" ht="38" customHeight="1">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="A43" s="9" t="inlineStr">
         <is>
           <t>oos</t>
         </is>
@@ -2741,7 +2749,7 @@
           <t>â€”</t>
         </is>
       </c>
-      <c r="I43" s="8" t="inlineStr">
+      <c r="I43" s="9" t="inlineStr">
         <is>
           <t>deferred</t>
         </is>

</xml_diff>

<commit_message>
﻿docs(roadmap): flip v1.0 rows 7, 9, 12 to completed
PRs #283 (Idle session timeout), #284 (DR runbook), and #285 (FR
completeness gate) are now on main (commit 26fe0a55) and uat
(commit ae06252d), so all three rows graduate from "started" to
"completed" per docs/roadmap.md status definition ("Shipped. The
deliverable described in the row is verifiable on the listed
branch").

Row 8 (Keycloak Phase C cutover) — its dependency (row 7) is now
completed and unblocked. Status remains "not-started" because the
cutover itself is a deployment toggle, not a code change.

Regenerated docs/roadmap.xlsx from the updated CSV — three rows now
render with the green "completed" tint.
</commit_message>
<xml_diff>
--- a/docs/roadmap.xlsx
+++ b/docs/roadmap.xlsx
@@ -33,7 +33,7 @@
       <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -58,11 +58,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFE699"/>
       </patternFill>
     </fill>
     <fill>
@@ -112,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -139,9 +134,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -877,9 +869,9 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>started</t>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>completed</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
@@ -981,9 +973,9 @@
           <t>Platform</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>started</t>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>completed</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
@@ -1137,9 +1129,9 @@
           <t>Frontend</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr">
-        <is>
-          <t>started</t>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>completed</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
@@ -1201,7 +1193,7 @@
       </c>
     </row>
     <row r="14" ht="38" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1253,7 +1245,7 @@
       </c>
     </row>
     <row r="15" ht="38" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1305,7 +1297,7 @@
       </c>
     </row>
     <row r="16" ht="38" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1357,7 +1349,7 @@
       </c>
     </row>
     <row r="17" ht="38" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1409,7 +1401,7 @@
       </c>
     </row>
     <row r="18" ht="38" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1461,7 +1453,7 @@
       </c>
     </row>
     <row r="19" ht="38" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1513,7 +1505,7 @@
       </c>
     </row>
     <row r="20" ht="38" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1565,7 +1557,7 @@
       </c>
     </row>
     <row r="21" ht="38" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1617,7 +1609,7 @@
       </c>
     </row>
     <row r="22" ht="38" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1669,7 +1661,7 @@
       </c>
     </row>
     <row r="23" ht="38" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1721,7 +1713,7 @@
       </c>
     </row>
     <row r="24" ht="38" customHeight="1">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1773,7 +1765,7 @@
       </c>
     </row>
     <row r="25" ht="38" customHeight="1">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1825,7 +1817,7 @@
       </c>
     </row>
     <row r="26" ht="38" customHeight="1">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>v1.1</t>
         </is>
@@ -1877,7 +1869,7 @@
       </c>
     </row>
     <row r="27" ht="38" customHeight="1">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -1929,7 +1921,7 @@
       </c>
     </row>
     <row r="28" ht="38" customHeight="1">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -1981,7 +1973,7 @@
       </c>
     </row>
     <row r="29" ht="38" customHeight="1">
-      <c r="A29" s="8" t="inlineStr">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -2033,7 +2025,7 @@
       </c>
     </row>
     <row r="30" ht="38" customHeight="1">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="A30" s="7" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -2085,7 +2077,7 @@
       </c>
     </row>
     <row r="31" ht="38" customHeight="1">
-      <c r="A31" s="8" t="inlineStr">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -2137,7 +2129,7 @@
       </c>
     </row>
     <row r="32" ht="38" customHeight="1">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -2189,7 +2181,7 @@
       </c>
     </row>
     <row r="33" ht="38" customHeight="1">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -2241,7 +2233,7 @@
       </c>
     </row>
     <row r="34" ht="38" customHeight="1">
-      <c r="A34" s="8" t="inlineStr">
+      <c r="A34" s="7" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -2293,7 +2285,7 @@
       </c>
     </row>
     <row r="35" ht="38" customHeight="1">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="A35" s="7" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -2345,7 +2337,7 @@
       </c>
     </row>
     <row r="36" ht="38" customHeight="1">
-      <c r="A36" s="8" t="inlineStr">
+      <c r="A36" s="7" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -2397,7 +2389,7 @@
       </c>
     </row>
     <row r="37" ht="38" customHeight="1">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="A37" s="7" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -2449,7 +2441,7 @@
       </c>
     </row>
     <row r="38" ht="38" customHeight="1">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="A38" s="7" t="inlineStr">
         <is>
           <t>v2.0</t>
         </is>
@@ -2501,7 +2493,7 @@
       </c>
     </row>
     <row r="39" ht="38" customHeight="1">
-      <c r="A39" s="9" t="inlineStr">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>oos</t>
         </is>
@@ -2541,7 +2533,7 @@
           <t>â€”</t>
         </is>
       </c>
-      <c r="I39" s="9" t="inlineStr">
+      <c r="I39" s="8" t="inlineStr">
         <is>
           <t>deferred</t>
         </is>
@@ -2553,7 +2545,7 @@
       </c>
     </row>
     <row r="40" ht="38" customHeight="1">
-      <c r="A40" s="9" t="inlineStr">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>oos</t>
         </is>
@@ -2593,7 +2585,7 @@
           <t>â€”</t>
         </is>
       </c>
-      <c r="I40" s="9" t="inlineStr">
+      <c r="I40" s="8" t="inlineStr">
         <is>
           <t>deferred</t>
         </is>
@@ -2605,7 +2597,7 @@
       </c>
     </row>
     <row r="41" ht="38" customHeight="1">
-      <c r="A41" s="9" t="inlineStr">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>oos</t>
         </is>
@@ -2645,7 +2637,7 @@
           <t>â€”</t>
         </is>
       </c>
-      <c r="I41" s="10" t="inlineStr">
+      <c r="I41" s="9" t="inlineStr">
         <is>
           <t>dropped</t>
         </is>
@@ -2657,7 +2649,7 @@
       </c>
     </row>
     <row r="42" ht="38" customHeight="1">
-      <c r="A42" s="9" t="inlineStr">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>oos</t>
         </is>
@@ -2697,7 +2689,7 @@
           <t>â€”</t>
         </is>
       </c>
-      <c r="I42" s="10" t="inlineStr">
+      <c r="I42" s="9" t="inlineStr">
         <is>
           <t>dropped</t>
         </is>
@@ -2709,7 +2701,7 @@
       </c>
     </row>
     <row r="43" ht="38" customHeight="1">
-      <c r="A43" s="9" t="inlineStr">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>oos</t>
         </is>
@@ -2749,7 +2741,7 @@
           <t>â€”</t>
         </is>
       </c>
-      <c r="I43" s="9" t="inlineStr">
+      <c r="I43" s="8" t="inlineStr">
         <is>
           <t>deferred</t>
         </is>

</xml_diff>

<commit_message>
docs(roadmap): regenerate roadmap.xlsx after rows 4/5/6/8 flip
The CSV is the source of truth; xlsx is a stakeholder-facing presentation
artifact (per docs/roadmap.md §How this roadmap is maintained). After
flipping rows 4 (T-68 offline dispense queue), 5 (T-71 Playwright E2E),
6 (T-72 perf baseline) and 8 (Keycloak Phase C cutover) to completed in
docs/roadmap.csv, the xlsx needs to be re-rendered so Excel/Numbers/
Sheets users see the same state.

Regenerated via the documented script:

  python3 -m venv /tmp/xlsx-venv && /tmp/xlsx-venv/bin/pip install -q openpyxl
  /tmp/xlsx-venv/bin/python scripts/build-roadmap-xlsx.py
  -> Wrote docs/roadmap.xlsx (42 rows)

Spot-checked: all twelve v1.0 rows show the expected status —
8 completed, 4 not-started (axe-core PR pending elsewhere; keyboard
nav blocked on axe-core; rc1 cut gates on every v1.0 row).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap.xlsx
+++ b/docs/roadmap.xlsx
@@ -596,7 +596,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -713,9 +713,9 @@
           <t>Mixed (Frontend + Backend)</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>completed</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -765,9 +765,9 @@
           <t>Frontend</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>completed</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -817,9 +817,9 @@
           <t>Platform</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>completed</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
@@ -856,7 +856,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -921,9 +921,9 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>completed</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>ORU^R01 â†’ LabResult persistence</t>
+          <t>ORU^R01 → LabResult persistence</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>ADT â†’ Admission/Encounter sync</t>
+          <t>ADT → Admission/Encounter sync</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1475,12 +1475,12 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Probabilistic match on name + DOB + sex + national-ID where present; candidate-match workflow in receptionist UI; â‰¥90% recall on labelled audit set</t>
+          <t>Probabilistic match on name + DOB + sex + national-ID where present; candidate-match workflow in receptionist UI; ≥90% recall on labelled audit set</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1636,7 +1636,7 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1792,7 +1792,7 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -1896,7 +1896,7 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -2094,17 +2094,17 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>SOC 2 Type I â†’ Type II</t>
+          <t>SOC 2 Type I → Type II</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Control map (existing audit logs/RBAC/encryption cover ~60% of CC1â€“CC9); gap analysis in docs/compliance/soc2-gap.md; 12-month observation window</t>
+          <t>Control map (existing audit logs/RBAC/encryption cover ~60% of CC1–CC9); gap analysis in docs/compliance/soc2-gap.md; 12-month observation window</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -2151,12 +2151,12 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>BAA template; PHI inventory; key rotation; access review cadence â€” for international customers</t>
+          <t>BAA template; PHI inventory; key rotation; access review cadence — for international customers</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -2203,12 +2203,12 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Per-tenant region pinning (Railway â†’ AWS or OVH-Africa); required for Senegal/CÃ´te d'Ivoire/Ghana sales</t>
+          <t>Per-tenant region pinning (Railway → AWS or OVH-Africa); required for Senegal/Côte d'Ivoire/Ghana sales</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -2312,7 +2312,7 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
@@ -2500,7 +2500,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -2515,22 +2515,22 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Deferred â€” regulatorily risky in healthcare; no existing groundwork in repo. Revisit after v1.0</t>
+          <t>Deferred — regulatorily risky in healthcare; no existing groundwork in repo. Revisit after v1.0</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I39" s="8" t="inlineStr">
@@ -2540,7 +2540,7 @@
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2552,7 +2552,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -2567,22 +2567,22 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Deferred â€” duplicates the OTelâ†’Grafana Cloud path landed in #276</t>
+          <t>Deferred — duplicates the OTel→Grafana Cloud path landed in #276</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I40" s="8" t="inlineStr">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2604,7 +2604,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -2619,22 +2619,22 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Dropped â€” GitHub Actions already covers CI/CD; Jenkins would be parallel duplication</t>
+          <t>Dropped — GitHub Actions already covers CI/CD; Jenkins would be parallel duplication</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I41" s="9" t="inlineStr">
@@ -2644,7 +2644,7 @@
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -2671,22 +2671,22 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Dropped â€” auth concerns belong in Keycloak; configure user federation there per deployment</t>
+          <t>Dropped — auth concerns belong in Keycloak; configure user federation there per deployment</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I42" s="9" t="inlineStr">
@@ -2696,7 +2696,7 @@
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2708,7 +2708,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -2723,22 +2723,22 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Deferred â€” out of scope for clinical+pharmacy MVP; partner with a billing vendor instead</t>
+          <t>Deferred — out of scope for clinical+pharmacy MVP; partner with a billing vendor instead</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I43" s="8" t="inlineStr">
@@ -2748,7 +2748,7 @@
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>â€”</t>
+          <t>—</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(roadmap): regenerate workbook after schema rebase
</commit_message>
<xml_diff>
--- a/docs/roadmap.xlsx
+++ b/docs/roadmap.xlsx
@@ -2211,7 +2211,7 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Row-level multi-tenancy stays default; schema-per-tenant available for hospitals with strong isolation needs (military, private foreign)</t>
+          <t>Row-level multi-tenancy stays default; schema-per-tenant available for hospitals with strong isolation needs (military, private foreign). Foundation pass landed on feat/v2.0-schema-per-tenant: TenantIsolationMode enum, Hospital.isolationMode + tenantSchemaName columns (V97 + CHECK constraints + partial unique index), SchemaTenantIdentifierResolver + SchemaTenantConnectionProvider + TenantSchemaLookup behind app.tenancy.schema-isolation.enabled (off by default), 28 unit tests, operational runbook docs/runbooks/schema-per-tenant-migration.md. Follow-on PRs: provision-schema.sh, copy-rows.sh, cache-invalidate endpoint.</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
@@ -2229,9 +2229,9 @@
           <t>Mixed (Backend + Platform)</t>
         </is>
       </c>
-      <c r="I33" s="5" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>started</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">

</xml_diff>

<commit_message>
chore(roadmap): flip rows 26/35/38 to started after overnight merges
PR #332 (row 24 ADT visit-sync) carried its own roadmap.csv update
on commit c07e439e — already in develop. This sync covers the
three other foundation passes that merged on 2026-05-16:

- Row 26 (CDS Hooks LOINC binding) — PR #333.
- Row 35 (Read replicas + Hikari tuning) — PR #334.
- Row 38 (HIPAA-equivalent posture) — PR #335.

Each row description rewritten in the same shape used for rows
23/24/33/37: deliverable headline + foundation-pass summary +
follow-on scope. roadmap.md gets a new 2026-05-16 narrative
blockquote naming the merge commits and the per-row "what shipped
vs what's deferred" lines. roadmap.xlsx regenerated from the CSV
via scripts/build-roadmap-xlsx.py (48 rows, status-tinted column).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap.xlsx
+++ b/docs/roadmap.xlsx
@@ -1743,7 +1743,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>ADT^A01/A04/A08 trigger Admission and Encounter sync; conflict-resolution rules documented</t>
+          <t>ADT^A01/A04/A08 trigger Admission and Encounter sync; conflict-resolution rules documented. Foundation pass shipped on feat/v1.1-adt-admission-encounter-sync (PR #332): V99 migration adds external_visit_number + external_sending_application + external_sending_facility + external_message_control_id (nullable) to admissions and clinical.encounters with partial composite unique indexes scoped per (sender, hospital); MllpInboundAdtVisitProjectionService reconciles inbound A01/A04/A08 against existing rows by the HL7 visit-number triplet, REQUIRES_NEW so projection failure cannot roll back the demographic write; gated behind app.hl7.adt.visit-sync.enabled (default false) so flag-off behaviour is bit-for-bit unchanged. Conflict-resolution rules + operator playbook in docs/runbooks/hl7-adt-conflict-resolution.md. Auto-create deferred to a follow-on PR (needs per-hospital intake-provider config).</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -1761,9 +1761,9 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="I24" s="7" t="inlineStr">
+        <is>
+          <t>started</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Bind hms-patient-view problem cards to LOINC alongside existing ICD</t>
+          <t>Bind hms-patient-view problem cards to LOINC alongside existing ICD. Shipped on feat/v1.1-cds-hooks-loinc-binding (PR #333): V100 migration adds loinc_code + loinc_display (nullable) to clinical.patient_problems; ProblemLoincBindings seed table (13 entries spanning cardio / endocrine / respiratory / hematology / malaria / HIV / TB / renal / OB â€” chosen for the WHO-EMRO chronic-care workload pilot hospitals see); PatientViewCdsService.renderProblem now appends typed [ICD-10: ...] and [LOINC: ...] annotations to each problem line, with entity-explicit loincCode taking precedence over the seed fallback. Malformed codes (failing TerminologyCodes regex) are dropped silently â€” card still renders, just without the annotation. 10 new tests cover prefix resolution, subdivision tolerance, case/whitespace, unknown codes, malformed input, and a defence-in-depth check that every seeded LOINC passes the global LOINC regex.</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -1865,9 +1865,9 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="I26" s="5" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="I26" s="7" t="inlineStr">
+        <is>
+          <t>started</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
@@ -2315,7 +2315,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Hikari pool sized to actual concurrent users; RO replica routing for FHIR reads and dashboards</t>
+          <t>Hikari pool sized to actual concurrent users; RO replica routing for FHIR reads and dashboards. Foundation pass shipped on feat/v2.0-read-replicas-hikari (PR #334): full Hikari tuning surface bound to spring.datasource.hikari.* (env-overridable pool-name / maximum-pool-size / minimum-idle / idle-timeout / max-lifetime / connection-timeout / leak-detection-threshold) â€” defaults sized for the documented Prod (single tenant) deployment. ReplicaDataSourceProperties (@ConfigurationProperties on app.datasource.replica.*) with fail-fast validation; ReadWriteRoutingDataSource extends AbstractRoutingDataSource and keys off TransactionSynchronizationManager.isCurrentTransactionReadOnly() (WRITE is the default â€” no txn, flag off, or missing replica all degrade to write). ReadReplicaDataSourceConfiguration is @ConditionalOnProperty-gated on app.datasource.replica.enabled. DataSourceConfig composes (write, optional replica) behind the routing wrapper; flag-off behaviour bit-for-bit unchanged. 11 unit tests cover routing-key derivation and replica fail-fast validation. Activation playbook + 5-business-day UAT soak procedure documented in docs/runbooks/postgres-pool-replica-sizing.md.</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
@@ -2333,9 +2333,9 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="I35" s="5" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>started</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>BAA template; PHI inventory; key rotation; access review cadence â€” for international customers</t>
+          <t>BAA template; PHI inventory; key rotation; access review cadence â€” for international customers. Foundation pass shipped on feat/v2.0-hipaa-posture (PR #335) â€” mirrors the SOC 2 row-37 pattern. docs/compliance/hipaa-gap.md inventories 51 control points across Â§164 Security Rule (administrative / physical / technical / organizational / docs) + Privacy Rule (minimum necessary + individual rights) â€” scorecard 19 present / 17 partial / 15 gap = 54% weighted, technical-safeguards axis at 75% (Â§164.312(a)(2)(iv) Encryption + Decryption rated partial: AES-256-GCM operational on 14 narrative columns via EncryptedStringConverter, identifier columns plaintext today). Companion machine-readable docs/compliance/hipaa-controls.csv + docs/compliance/hipaa-baa-template.md (11-section BAA draft with sub-BAA table for Railway / Splunk / Grafana / Keycloak host / email + SMS vendors) + docs/compliance/phi-inventory.md (all 18 Â§164.514(b)(2) identifier categories + clinical-record body, per-column encryption status, dataflow map). 27-item remediation backlog (10 P0 / 10 P1 / 7 P2); P0 critical path 2026-09-30 calibrated to land one month after the SOC 2 P0 deadline.</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
@@ -2489,9 +2489,9 @@
           <t>Compliance</t>
         </is>
       </c>
-      <c r="I38" s="5" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="I38" s="7" t="inlineStr">
+        <is>
+          <t>started</t>
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr">

</xml_diff>